<commit_message>
Roster template v2: fitted cells, manpower table, shift times, tight legend, one-page print certified
</commit_message>
<xml_diff>
--- a/uploads/inbox/SPV_CABIN_ROSTER_TEMPLATE.xlsx
+++ b/uploads/inbox/SPV_CABIN_ROSTER_TEMPLATE.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROSTER" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROSTER'!$A$1:$AI$60</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROSTER'!$A$1:$AI$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,11 +30,7 @@
     <font>
       <b val="1"/>
       <color rgb="00196B24"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -42,17 +38,7 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00B45309"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E3D"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -60,15 +46,52 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00B45309"/>
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="008A9299"/>
-      <sz val="8"/>
+      <b val="1"/>
+      <color rgb="001F4E3D"/>
+      <sz val="10"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <color rgb="009AA2A9"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A56DB"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
@@ -81,9 +104,6 @@
       <sz val="9"/>
     </font>
     <font>
-      <sz val="8"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="001A56DB"/>
       <sz val="9"/>
@@ -94,59 +114,66 @@
       <sz val="9"/>
     </font>
     <font>
+      <sz val="7"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="005521B5"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="000E7490"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="006B7280"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00F9FAFB"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="007E22CE"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00C2410C"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="003730A3"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00BE123C"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="003F6212"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00475569"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00713F12"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="7"/>
     </font>
   </fonts>
   <fills count="21">
@@ -252,7 +279,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -275,16 +302,84 @@
       </bottom>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9CFD6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CFD6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CFD6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CFD6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CFD6"/>
+      </top>
       <bottom style="thin">
-        <color rgb="004A5560"/>
+        <color rgb="00C9CFD6"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9CFD6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CFD6"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9CFD6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9CFD6"/>
+      </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="004A5560"/>
+        <color rgb="00C9CFD6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CFD6"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9CFD6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -292,59 +387,63 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -352,41 +451,66 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -396,7 +520,7 @@
       <font>
         <b val="1"/>
         <color rgb="0092400E"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -408,7 +532,7 @@
       <font>
         <b val="1"/>
         <color rgb="001A56DB"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -420,7 +544,7 @@
       <font>
         <b val="1"/>
         <color rgb="00065F46"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -432,7 +556,7 @@
       <font>
         <b val="1"/>
         <color rgb="005521B5"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -444,7 +568,7 @@
       <font>
         <b val="1"/>
         <color rgb="000E7490"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -456,7 +580,7 @@
       <font>
         <b val="1"/>
         <color rgb="006B7280"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -468,7 +592,7 @@
       <font>
         <b val="1"/>
         <color rgb="00F9FAFB"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -480,7 +604,7 @@
       <font>
         <b val="1"/>
         <color rgb="007E22CE"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -492,7 +616,7 @@
       <font>
         <b val="1"/>
         <color rgb="00C2410C"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -504,7 +628,7 @@
       <font>
         <b val="1"/>
         <color rgb="003730A3"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -516,7 +640,7 @@
       <font>
         <b val="1"/>
         <color rgb="00BE123C"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -528,7 +652,7 @@
       <font>
         <b val="1"/>
         <color rgb="003F6212"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -540,7 +664,7 @@
       <font>
         <b val="1"/>
         <color rgb="00475569"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -552,7 +676,7 @@
       <font>
         <b val="1"/>
         <color rgb="00713F12"/>
-        <sz val="9"/>
+        <sz val="8.5"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -927,50 +1051,50 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK59"/>
+  <dimension ref="A1:AK60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3.5" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="9.5" customWidth="1" min="4" max="4"/>
-    <col width="3.4" customWidth="1" min="5" max="5"/>
-    <col width="3.4" customWidth="1" min="6" max="6"/>
-    <col width="3.4" customWidth="1" min="7" max="7"/>
-    <col width="3.4" customWidth="1" min="8" max="8"/>
-    <col width="3.4" customWidth="1" min="9" max="9"/>
-    <col width="3.4" customWidth="1" min="10" max="10"/>
-    <col width="3.4" customWidth="1" min="11" max="11"/>
-    <col width="3.4" customWidth="1" min="12" max="12"/>
-    <col width="3.4" customWidth="1" min="13" max="13"/>
-    <col width="3.4" customWidth="1" min="14" max="14"/>
-    <col width="3.4" customWidth="1" min="15" max="15"/>
-    <col width="3.4" customWidth="1" min="16" max="16"/>
-    <col width="3.4" customWidth="1" min="17" max="17"/>
-    <col width="3.4" customWidth="1" min="18" max="18"/>
-    <col width="3.4" customWidth="1" min="19" max="19"/>
-    <col width="3.4" customWidth="1" min="20" max="20"/>
-    <col width="3.4" customWidth="1" min="21" max="21"/>
-    <col width="3.4" customWidth="1" min="22" max="22"/>
-    <col width="3.4" customWidth="1" min="23" max="23"/>
-    <col width="3.4" customWidth="1" min="24" max="24"/>
-    <col width="3.4" customWidth="1" min="25" max="25"/>
-    <col width="3.4" customWidth="1" min="26" max="26"/>
-    <col width="3.4" customWidth="1" min="27" max="27"/>
-    <col width="3.4" customWidth="1" min="28" max="28"/>
-    <col width="3.4" customWidth="1" min="29" max="29"/>
-    <col width="3.4" customWidth="1" min="30" max="30"/>
-    <col width="3.4" customWidth="1" min="31" max="31"/>
-    <col width="3.4" customWidth="1" min="32" max="32"/>
-    <col width="3.4" customWidth="1" min="33" max="33"/>
-    <col width="3.4" customWidth="1" min="34" max="34"/>
-    <col width="3.4" customWidth="1" min="35" max="35"/>
+    <col width="6.4" customWidth="1" min="1" max="1"/>
+    <col width="9.5" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="8.800000000000001" customWidth="1" min="4" max="4"/>
+    <col width="3.5" customWidth="1" min="5" max="5"/>
+    <col width="3.5" customWidth="1" min="6" max="6"/>
+    <col width="3.5" customWidth="1" min="7" max="7"/>
+    <col width="3.5" customWidth="1" min="8" max="8"/>
+    <col width="3.5" customWidth="1" min="9" max="9"/>
+    <col width="3.5" customWidth="1" min="10" max="10"/>
+    <col width="3.5" customWidth="1" min="11" max="11"/>
+    <col width="3.5" customWidth="1" min="12" max="12"/>
+    <col width="3.5" customWidth="1" min="13" max="13"/>
+    <col width="3.5" customWidth="1" min="14" max="14"/>
+    <col width="3.5" customWidth="1" min="15" max="15"/>
+    <col width="3.5" customWidth="1" min="16" max="16"/>
+    <col width="3.5" customWidth="1" min="17" max="17"/>
+    <col width="3.5" customWidth="1" min="18" max="18"/>
+    <col width="3.5" customWidth="1" min="19" max="19"/>
+    <col width="3.5" customWidth="1" min="20" max="20"/>
+    <col width="3.5" customWidth="1" min="21" max="21"/>
+    <col width="3.5" customWidth="1" min="22" max="22"/>
+    <col width="3.5" customWidth="1" min="23" max="23"/>
+    <col width="3.5" customWidth="1" min="24" max="24"/>
+    <col width="3.5" customWidth="1" min="25" max="25"/>
+    <col width="3.5" customWidth="1" min="26" max="26"/>
+    <col width="3.5" customWidth="1" min="27" max="27"/>
+    <col width="3.5" customWidth="1" min="28" max="28"/>
+    <col width="3.5" customWidth="1" min="29" max="29"/>
+    <col width="3.5" customWidth="1" min="30" max="30"/>
+    <col width="3.5" customWidth="1" min="31" max="31"/>
+    <col width="3.5" customWidth="1" min="32" max="32"/>
+    <col width="3.5" customWidth="1" min="33" max="33"/>
+    <col width="3.5" customWidth="1" min="34" max="34"/>
+    <col width="3.5" customWidth="1" min="35" max="35"/>
     <col hidden="1" width="13" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SAUDIA TECHNIC</t>
@@ -981,16 +1105,16 @@
           <t>AIRCRAFT HEAVY MAINTENANCE · SPV CABIN — MONTHLY ROSTER</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="AF1" s="3" t="inlineStr">
         <is>
           <t>CC: 264</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>MONTH:</t>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="42" t="inlineStr">
+        <is>
+          <t>MONTH</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1000,7 +1124,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>YEAR:</t>
+          <t>YEAR</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
@@ -1015,7 +1139,7 @@
         <v/>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="12" customHeight="1">
       <c r="E3" s="7">
         <f>IF(1&lt;=DAY(EOMONTH(DATE($D$2,$AK$2,1),0)),TEXT(DATE($D$2,$AK$2,1),"ddd"),"")</f>
         <v/>
@@ -1141,7 +1265,7 @@
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="14" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>#</t>
@@ -1287,7 +1411,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>CREW 1</t>
@@ -1325,7 +1449,7 @@
       <c r="AH5" s="10" t="n"/>
       <c r="AI5" s="10" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="14.5" customHeight="1">
       <c r="A6" s="11" t="n">
         <v>1</v>
       </c>
@@ -1364,7 +1488,7 @@
       <c r="AH6" s="13" t="n"/>
       <c r="AI6" s="13" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14.5" customHeight="1">
       <c r="A7" s="11" t="n">
         <v>2</v>
       </c>
@@ -1403,7 +1527,7 @@
       <c r="AH7" s="13" t="n"/>
       <c r="AI7" s="13" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="14.5" customHeight="1">
       <c r="A8" s="11" t="n">
         <v>3</v>
       </c>
@@ -1442,7 +1566,7 @@
       <c r="AH8" s="13" t="n"/>
       <c r="AI8" s="13" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="14.5" customHeight="1">
       <c r="A9" s="11" t="n">
         <v>4</v>
       </c>
@@ -1481,7 +1605,7 @@
       <c r="AH9" s="13" t="n"/>
       <c r="AI9" s="13" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="14.5" customHeight="1">
       <c r="A10" s="11" t="n">
         <v>5</v>
       </c>
@@ -1520,7 +1644,7 @@
       <c r="AH10" s="13" t="n"/>
       <c r="AI10" s="13" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="14.5" customHeight="1">
       <c r="A11" s="11" t="n">
         <v>6</v>
       </c>
@@ -1559,7 +1683,7 @@
       <c r="AH11" s="13" t="n"/>
       <c r="AI11" s="13" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="14.5" customHeight="1">
       <c r="A12" s="11" t="n">
         <v>7</v>
       </c>
@@ -1598,7 +1722,7 @@
       <c r="AH12" s="13" t="n"/>
       <c r="AI12" s="13" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="14.5" customHeight="1">
       <c r="A13" s="11" t="n">
         <v>8</v>
       </c>
@@ -1637,7 +1761,7 @@
       <c r="AH13" s="13" t="n"/>
       <c r="AI13" s="13" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="14.5" customHeight="1">
       <c r="A14" s="11" t="n">
         <v>9</v>
       </c>
@@ -1676,7 +1800,7 @@
       <c r="AH14" s="13" t="n"/>
       <c r="AI14" s="13" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="14.5" customHeight="1">
       <c r="A15" s="11" t="n">
         <v>10</v>
       </c>
@@ -1715,7 +1839,7 @@
       <c r="AH15" s="13" t="n"/>
       <c r="AI15" s="13" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="14.5" customHeight="1">
       <c r="A16" s="11" t="n">
         <v>11</v>
       </c>
@@ -1754,7 +1878,7 @@
       <c r="AH16" s="13" t="n"/>
       <c r="AI16" s="13" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="14.5" customHeight="1">
       <c r="A17" s="11" t="n">
         <v>12</v>
       </c>
@@ -1793,47 +1917,86 @@
       <c r="AH17" s="13" t="n"/>
       <c r="AI17" s="13" t="n"/>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>CREW 2</t>
         </is>
       </c>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="15" t="n"/>
-      <c r="I19" s="15" t="n"/>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
-      <c r="L19" s="15" t="n"/>
-      <c r="M19" s="15" t="n"/>
-      <c r="N19" s="15" t="n"/>
-      <c r="O19" s="15" t="n"/>
-      <c r="P19" s="15" t="n"/>
-      <c r="Q19" s="15" t="n"/>
-      <c r="R19" s="15" t="n"/>
-      <c r="S19" s="15" t="n"/>
-      <c r="T19" s="15" t="n"/>
-      <c r="U19" s="15" t="n"/>
-      <c r="V19" s="15" t="n"/>
-      <c r="W19" s="15" t="n"/>
-      <c r="X19" s="15" t="n"/>
-      <c r="Y19" s="15" t="n"/>
-      <c r="Z19" s="15" t="n"/>
-      <c r="AA19" s="15" t="n"/>
-      <c r="AB19" s="15" t="n"/>
-      <c r="AC19" s="15" t="n"/>
-      <c r="AD19" s="15" t="n"/>
-      <c r="AE19" s="15" t="n"/>
-      <c r="AF19" s="15" t="n"/>
-      <c r="AG19" s="15" t="n"/>
-      <c r="AH19" s="15" t="n"/>
-      <c r="AI19" s="15" t="n"/>
-    </row>
-    <row r="20">
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="15" t="n"/>
+      <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="15" t="n"/>
+      <c r="S18" s="15" t="n"/>
+      <c r="T18" s="15" t="n"/>
+      <c r="U18" s="15" t="n"/>
+      <c r="V18" s="15" t="n"/>
+      <c r="W18" s="15" t="n"/>
+      <c r="X18" s="15" t="n"/>
+      <c r="Y18" s="15" t="n"/>
+      <c r="Z18" s="15" t="n"/>
+      <c r="AA18" s="15" t="n"/>
+      <c r="AB18" s="15" t="n"/>
+      <c r="AC18" s="15" t="n"/>
+      <c r="AD18" s="15" t="n"/>
+      <c r="AE18" s="15" t="n"/>
+      <c r="AF18" s="15" t="n"/>
+      <c r="AG18" s="15" t="n"/>
+      <c r="AH18" s="15" t="n"/>
+      <c r="AI18" s="15" t="n"/>
+    </row>
+    <row r="19" ht="14.5" customHeight="1">
+      <c r="A19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="13" t="n"/>
+      <c r="M19" s="13" t="n"/>
+      <c r="N19" s="13" t="n"/>
+      <c r="O19" s="13" t="n"/>
+      <c r="P19" s="13" t="n"/>
+      <c r="Q19" s="13" t="n"/>
+      <c r="R19" s="13" t="n"/>
+      <c r="S19" s="13" t="n"/>
+      <c r="T19" s="13" t="n"/>
+      <c r="U19" s="13" t="n"/>
+      <c r="V19" s="13" t="n"/>
+      <c r="W19" s="13" t="n"/>
+      <c r="X19" s="13" t="n"/>
+      <c r="Y19" s="13" t="n"/>
+      <c r="Z19" s="13" t="n"/>
+      <c r="AA19" s="13" t="n"/>
+      <c r="AB19" s="13" t="n"/>
+      <c r="AC19" s="13" t="n"/>
+      <c r="AD19" s="13" t="n"/>
+      <c r="AE19" s="13" t="n"/>
+      <c r="AF19" s="13" t="n"/>
+      <c r="AG19" s="13" t="n"/>
+      <c r="AH19" s="13" t="n"/>
+      <c r="AI19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="14.5" customHeight="1">
       <c r="A20" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B20" s="11" t="n"/>
       <c r="C20" s="12" t="n"/>
@@ -1870,9 +2033,9 @@
       <c r="AH20" s="13" t="n"/>
       <c r="AI20" s="13" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" ht="14.5" customHeight="1">
       <c r="A21" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B21" s="11" t="n"/>
       <c r="C21" s="12" t="n"/>
@@ -1909,9 +2072,9 @@
       <c r="AH21" s="13" t="n"/>
       <c r="AI21" s="13" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="14.5" customHeight="1">
       <c r="A22" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B22" s="11" t="n"/>
       <c r="C22" s="12" t="n"/>
@@ -1948,9 +2111,9 @@
       <c r="AH22" s="13" t="n"/>
       <c r="AI22" s="13" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" ht="14.5" customHeight="1">
       <c r="A23" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B23" s="11" t="n"/>
       <c r="C23" s="12" t="n"/>
@@ -1987,9 +2150,9 @@
       <c r="AH23" s="13" t="n"/>
       <c r="AI23" s="13" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" ht="14.5" customHeight="1">
       <c r="A24" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B24" s="11" t="n"/>
       <c r="C24" s="12" t="n"/>
@@ -2026,9 +2189,9 @@
       <c r="AH24" s="13" t="n"/>
       <c r="AI24" s="13" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="14.5" customHeight="1">
       <c r="A25" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B25" s="11" t="n"/>
       <c r="C25" s="12" t="n"/>
@@ -2065,9 +2228,9 @@
       <c r="AH25" s="13" t="n"/>
       <c r="AI25" s="13" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" ht="14.5" customHeight="1">
       <c r="A26" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="12" t="n"/>
@@ -2104,9 +2267,9 @@
       <c r="AH26" s="13" t="n"/>
       <c r="AI26" s="13" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="14.5" customHeight="1">
       <c r="A27" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B27" s="11" t="n"/>
       <c r="C27" s="12" t="n"/>
@@ -2143,9 +2306,9 @@
       <c r="AH27" s="13" t="n"/>
       <c r="AI27" s="13" t="n"/>
     </row>
-    <row r="28">
+    <row r="28" ht="14.5" customHeight="1">
       <c r="A28" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B28" s="11" t="n"/>
       <c r="C28" s="12" t="n"/>
@@ -2182,9 +2345,9 @@
       <c r="AH28" s="13" t="n"/>
       <c r="AI28" s="13" t="n"/>
     </row>
-    <row r="29">
+    <row r="29" ht="14.5" customHeight="1">
       <c r="A29" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B29" s="11" t="n"/>
       <c r="C29" s="12" t="n"/>
@@ -2221,9 +2384,9 @@
       <c r="AH29" s="13" t="n"/>
       <c r="AI29" s="13" t="n"/>
     </row>
-    <row r="30">
+    <row r="30" ht="14.5" customHeight="1">
       <c r="A30" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B30" s="11" t="n"/>
       <c r="C30" s="12" t="n"/>
@@ -2260,86 +2423,125 @@
       <c r="AH30" s="13" t="n"/>
       <c r="AI30" s="13" t="n"/>
     </row>
-    <row r="31">
-      <c r="A31" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="12" t="n"/>
-      <c r="D31" s="11" t="n"/>
-      <c r="E31" s="13" t="n"/>
-      <c r="F31" s="13" t="n"/>
-      <c r="G31" s="13" t="n"/>
-      <c r="H31" s="13" t="n"/>
-      <c r="I31" s="13" t="n"/>
-      <c r="J31" s="13" t="n"/>
-      <c r="K31" s="13" t="n"/>
-      <c r="L31" s="13" t="n"/>
-      <c r="M31" s="13" t="n"/>
-      <c r="N31" s="13" t="n"/>
-      <c r="O31" s="13" t="n"/>
-      <c r="P31" s="13" t="n"/>
-      <c r="Q31" s="13" t="n"/>
-      <c r="R31" s="13" t="n"/>
-      <c r="S31" s="13" t="n"/>
-      <c r="T31" s="13" t="n"/>
-      <c r="U31" s="13" t="n"/>
-      <c r="V31" s="13" t="n"/>
-      <c r="W31" s="13" t="n"/>
-      <c r="X31" s="13" t="n"/>
-      <c r="Y31" s="13" t="n"/>
-      <c r="Z31" s="13" t="n"/>
-      <c r="AA31" s="13" t="n"/>
-      <c r="AB31" s="13" t="n"/>
-      <c r="AC31" s="13" t="n"/>
-      <c r="AD31" s="13" t="n"/>
-      <c r="AE31" s="13" t="n"/>
-      <c r="AF31" s="13" t="n"/>
-      <c r="AG31" s="13" t="n"/>
-      <c r="AH31" s="13" t="n"/>
-      <c r="AI31" s="13" t="n"/>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>CREW 3</t>
         </is>
       </c>
-      <c r="E33" s="17" t="n"/>
-      <c r="F33" s="17" t="n"/>
-      <c r="G33" s="17" t="n"/>
-      <c r="H33" s="17" t="n"/>
-      <c r="I33" s="17" t="n"/>
-      <c r="J33" s="17" t="n"/>
-      <c r="K33" s="17" t="n"/>
-      <c r="L33" s="17" t="n"/>
-      <c r="M33" s="17" t="n"/>
-      <c r="N33" s="17" t="n"/>
-      <c r="O33" s="17" t="n"/>
-      <c r="P33" s="17" t="n"/>
-      <c r="Q33" s="17" t="n"/>
-      <c r="R33" s="17" t="n"/>
-      <c r="S33" s="17" t="n"/>
-      <c r="T33" s="17" t="n"/>
-      <c r="U33" s="17" t="n"/>
-      <c r="V33" s="17" t="n"/>
-      <c r="W33" s="17" t="n"/>
-      <c r="X33" s="17" t="n"/>
-      <c r="Y33" s="17" t="n"/>
-      <c r="Z33" s="17" t="n"/>
-      <c r="AA33" s="17" t="n"/>
-      <c r="AB33" s="17" t="n"/>
-      <c r="AC33" s="17" t="n"/>
-      <c r="AD33" s="17" t="n"/>
-      <c r="AE33" s="17" t="n"/>
-      <c r="AF33" s="17" t="n"/>
-      <c r="AG33" s="17" t="n"/>
-      <c r="AH33" s="17" t="n"/>
-      <c r="AI33" s="17" t="n"/>
-    </row>
-    <row r="34">
+      <c r="E31" s="17" t="n"/>
+      <c r="F31" s="17" t="n"/>
+      <c r="G31" s="17" t="n"/>
+      <c r="H31" s="17" t="n"/>
+      <c r="I31" s="17" t="n"/>
+      <c r="J31" s="17" t="n"/>
+      <c r="K31" s="17" t="n"/>
+      <c r="L31" s="17" t="n"/>
+      <c r="M31" s="17" t="n"/>
+      <c r="N31" s="17" t="n"/>
+      <c r="O31" s="17" t="n"/>
+      <c r="P31" s="17" t="n"/>
+      <c r="Q31" s="17" t="n"/>
+      <c r="R31" s="17" t="n"/>
+      <c r="S31" s="17" t="n"/>
+      <c r="T31" s="17" t="n"/>
+      <c r="U31" s="17" t="n"/>
+      <c r="V31" s="17" t="n"/>
+      <c r="W31" s="17" t="n"/>
+      <c r="X31" s="17" t="n"/>
+      <c r="Y31" s="17" t="n"/>
+      <c r="Z31" s="17" t="n"/>
+      <c r="AA31" s="17" t="n"/>
+      <c r="AB31" s="17" t="n"/>
+      <c r="AC31" s="17" t="n"/>
+      <c r="AD31" s="17" t="n"/>
+      <c r="AE31" s="17" t="n"/>
+      <c r="AF31" s="17" t="n"/>
+      <c r="AG31" s="17" t="n"/>
+      <c r="AH31" s="17" t="n"/>
+      <c r="AI31" s="17" t="n"/>
+    </row>
+    <row r="32" ht="14.5" customHeight="1">
+      <c r="A32" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="13" t="n"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="n"/>
+      <c r="J32" s="13" t="n"/>
+      <c r="K32" s="13" t="n"/>
+      <c r="L32" s="13" t="n"/>
+      <c r="M32" s="13" t="n"/>
+      <c r="N32" s="13" t="n"/>
+      <c r="O32" s="13" t="n"/>
+      <c r="P32" s="13" t="n"/>
+      <c r="Q32" s="13" t="n"/>
+      <c r="R32" s="13" t="n"/>
+      <c r="S32" s="13" t="n"/>
+      <c r="T32" s="13" t="n"/>
+      <c r="U32" s="13" t="n"/>
+      <c r="V32" s="13" t="n"/>
+      <c r="W32" s="13" t="n"/>
+      <c r="X32" s="13" t="n"/>
+      <c r="Y32" s="13" t="n"/>
+      <c r="Z32" s="13" t="n"/>
+      <c r="AA32" s="13" t="n"/>
+      <c r="AB32" s="13" t="n"/>
+      <c r="AC32" s="13" t="n"/>
+      <c r="AD32" s="13" t="n"/>
+      <c r="AE32" s="13" t="n"/>
+      <c r="AF32" s="13" t="n"/>
+      <c r="AG32" s="13" t="n"/>
+      <c r="AH32" s="13" t="n"/>
+      <c r="AI32" s="13" t="n"/>
+    </row>
+    <row r="33" ht="14.5" customHeight="1">
+      <c r="A33" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="13" t="n"/>
+      <c r="F33" s="13" t="n"/>
+      <c r="G33" s="13" t="n"/>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="13" t="n"/>
+      <c r="J33" s="13" t="n"/>
+      <c r="K33" s="13" t="n"/>
+      <c r="L33" s="13" t="n"/>
+      <c r="M33" s="13" t="n"/>
+      <c r="N33" s="13" t="n"/>
+      <c r="O33" s="13" t="n"/>
+      <c r="P33" s="13" t="n"/>
+      <c r="Q33" s="13" t="n"/>
+      <c r="R33" s="13" t="n"/>
+      <c r="S33" s="13" t="n"/>
+      <c r="T33" s="13" t="n"/>
+      <c r="U33" s="13" t="n"/>
+      <c r="V33" s="13" t="n"/>
+      <c r="W33" s="13" t="n"/>
+      <c r="X33" s="13" t="n"/>
+      <c r="Y33" s="13" t="n"/>
+      <c r="Z33" s="13" t="n"/>
+      <c r="AA33" s="13" t="n"/>
+      <c r="AB33" s="13" t="n"/>
+      <c r="AC33" s="13" t="n"/>
+      <c r="AD33" s="13" t="n"/>
+      <c r="AE33" s="13" t="n"/>
+      <c r="AF33" s="13" t="n"/>
+      <c r="AG33" s="13" t="n"/>
+      <c r="AH33" s="13" t="n"/>
+      <c r="AI33" s="13" t="n"/>
+    </row>
+    <row r="34" ht="14.5" customHeight="1">
       <c r="A34" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B34" s="11" t="n"/>
       <c r="C34" s="12" t="n"/>
@@ -2376,9 +2578,9 @@
       <c r="AH34" s="13" t="n"/>
       <c r="AI34" s="13" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" ht="14.5" customHeight="1">
       <c r="A35" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B35" s="11" t="n"/>
       <c r="C35" s="12" t="n"/>
@@ -2415,9 +2617,9 @@
       <c r="AH35" s="13" t="n"/>
       <c r="AI35" s="13" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="14.5" customHeight="1">
       <c r="A36" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B36" s="11" t="n"/>
       <c r="C36" s="12" t="n"/>
@@ -2454,9 +2656,9 @@
       <c r="AH36" s="13" t="n"/>
       <c r="AI36" s="13" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" ht="14.5" customHeight="1">
       <c r="A37" s="11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B37" s="11" t="n"/>
       <c r="C37" s="12" t="n"/>
@@ -2493,9 +2695,9 @@
       <c r="AH37" s="13" t="n"/>
       <c r="AI37" s="13" t="n"/>
     </row>
-    <row r="38">
+    <row r="38" ht="14.5" customHeight="1">
       <c r="A38" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B38" s="11" t="n"/>
       <c r="C38" s="12" t="n"/>
@@ -2532,9 +2734,9 @@
       <c r="AH38" s="13" t="n"/>
       <c r="AI38" s="13" t="n"/>
     </row>
-    <row r="39">
+    <row r="39" ht="14.5" customHeight="1">
       <c r="A39" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B39" s="11" t="n"/>
       <c r="C39" s="12" t="n"/>
@@ -2571,9 +2773,9 @@
       <c r="AH39" s="13" t="n"/>
       <c r="AI39" s="13" t="n"/>
     </row>
-    <row r="40">
+    <row r="40" ht="14.5" customHeight="1">
       <c r="A40" s="11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B40" s="11" t="n"/>
       <c r="C40" s="12" t="n"/>
@@ -2610,9 +2812,9 @@
       <c r="AH40" s="13" t="n"/>
       <c r="AI40" s="13" t="n"/>
     </row>
-    <row r="41">
+    <row r="41" ht="14.5" customHeight="1">
       <c r="A41" s="11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B41" s="11" t="n"/>
       <c r="C41" s="12" t="n"/>
@@ -2649,9 +2851,9 @@
       <c r="AH41" s="13" t="n"/>
       <c r="AI41" s="13" t="n"/>
     </row>
-    <row r="42">
+    <row r="42" ht="14.5" customHeight="1">
       <c r="A42" s="11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B42" s="11" t="n"/>
       <c r="C42" s="12" t="n"/>
@@ -2688,9 +2890,9 @@
       <c r="AH42" s="13" t="n"/>
       <c r="AI42" s="13" t="n"/>
     </row>
-    <row r="43">
+    <row r="43" ht="14.5" customHeight="1">
       <c r="A43" s="11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B43" s="11" t="n"/>
       <c r="C43" s="12" t="n"/>
@@ -2727,48 +2929,47 @@
       <c r="AH43" s="13" t="n"/>
       <c r="AI43" s="13" t="n"/>
     </row>
-    <row r="44">
-      <c r="A44" s="11" t="n">
-        <v>11</v>
-      </c>
-      <c r="B44" s="11" t="n"/>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="11" t="n"/>
-      <c r="E44" s="13" t="n"/>
-      <c r="F44" s="13" t="n"/>
-      <c r="G44" s="13" t="n"/>
-      <c r="H44" s="13" t="n"/>
-      <c r="I44" s="13" t="n"/>
-      <c r="J44" s="13" t="n"/>
-      <c r="K44" s="13" t="n"/>
-      <c r="L44" s="13" t="n"/>
-      <c r="M44" s="13" t="n"/>
-      <c r="N44" s="13" t="n"/>
-      <c r="O44" s="13" t="n"/>
-      <c r="P44" s="13" t="n"/>
-      <c r="Q44" s="13" t="n"/>
-      <c r="R44" s="13" t="n"/>
-      <c r="S44" s="13" t="n"/>
-      <c r="T44" s="13" t="n"/>
-      <c r="U44" s="13" t="n"/>
-      <c r="V44" s="13" t="n"/>
-      <c r="W44" s="13" t="n"/>
-      <c r="X44" s="13" t="n"/>
-      <c r="Y44" s="13" t="n"/>
-      <c r="Z44" s="13" t="n"/>
-      <c r="AA44" s="13" t="n"/>
-      <c r="AB44" s="13" t="n"/>
-      <c r="AC44" s="13" t="n"/>
-      <c r="AD44" s="13" t="n"/>
-      <c r="AE44" s="13" t="n"/>
-      <c r="AF44" s="13" t="n"/>
-      <c r="AG44" s="13" t="n"/>
-      <c r="AH44" s="13" t="n"/>
-      <c r="AI44" s="13" t="n"/>
-    </row>
-    <row r="45">
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>SPECIAL SHIFTING</t>
+        </is>
+      </c>
+      <c r="E44" s="19" t="n"/>
+      <c r="F44" s="19" t="n"/>
+      <c r="G44" s="19" t="n"/>
+      <c r="H44" s="19" t="n"/>
+      <c r="I44" s="19" t="n"/>
+      <c r="J44" s="19" t="n"/>
+      <c r="K44" s="19" t="n"/>
+      <c r="L44" s="19" t="n"/>
+      <c r="M44" s="19" t="n"/>
+      <c r="N44" s="19" t="n"/>
+      <c r="O44" s="19" t="n"/>
+      <c r="P44" s="19" t="n"/>
+      <c r="Q44" s="19" t="n"/>
+      <c r="R44" s="19" t="n"/>
+      <c r="S44" s="19" t="n"/>
+      <c r="T44" s="19" t="n"/>
+      <c r="U44" s="19" t="n"/>
+      <c r="V44" s="19" t="n"/>
+      <c r="W44" s="19" t="n"/>
+      <c r="X44" s="19" t="n"/>
+      <c r="Y44" s="19" t="n"/>
+      <c r="Z44" s="19" t="n"/>
+      <c r="AA44" s="19" t="n"/>
+      <c r="AB44" s="19" t="n"/>
+      <c r="AC44" s="19" t="n"/>
+      <c r="AD44" s="19" t="n"/>
+      <c r="AE44" s="19" t="n"/>
+      <c r="AF44" s="19" t="n"/>
+      <c r="AG44" s="19" t="n"/>
+      <c r="AH44" s="19" t="n"/>
+      <c r="AI44" s="19" t="n"/>
+    </row>
+    <row r="45" ht="14.5" customHeight="1">
       <c r="A45" s="11" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B45" s="11" t="n"/>
       <c r="C45" s="12" t="n"/>
@@ -2805,47 +3006,87 @@
       <c r="AH45" s="13" t="n"/>
       <c r="AI45" s="13" t="n"/>
     </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="18" t="inlineStr">
-        <is>
-          <t>SPECIAL SHIFTING</t>
-        </is>
-      </c>
-      <c r="E47" s="19" t="n"/>
-      <c r="F47" s="19" t="n"/>
-      <c r="G47" s="19" t="n"/>
-      <c r="H47" s="19" t="n"/>
-      <c r="I47" s="19" t="n"/>
-      <c r="J47" s="19" t="n"/>
-      <c r="K47" s="19" t="n"/>
-      <c r="L47" s="19" t="n"/>
-      <c r="M47" s="19" t="n"/>
-      <c r="N47" s="19" t="n"/>
-      <c r="O47" s="19" t="n"/>
-      <c r="P47" s="19" t="n"/>
-      <c r="Q47" s="19" t="n"/>
-      <c r="R47" s="19" t="n"/>
-      <c r="S47" s="19" t="n"/>
-      <c r="T47" s="19" t="n"/>
-      <c r="U47" s="19" t="n"/>
-      <c r="V47" s="19" t="n"/>
-      <c r="W47" s="19" t="n"/>
-      <c r="X47" s="19" t="n"/>
-      <c r="Y47" s="19" t="n"/>
-      <c r="Z47" s="19" t="n"/>
-      <c r="AA47" s="19" t="n"/>
-      <c r="AB47" s="19" t="n"/>
-      <c r="AC47" s="19" t="n"/>
-      <c r="AD47" s="19" t="n"/>
-      <c r="AE47" s="19" t="n"/>
-      <c r="AF47" s="19" t="n"/>
-      <c r="AG47" s="19" t="n"/>
-      <c r="AH47" s="19" t="n"/>
-      <c r="AI47" s="19" t="n"/>
-    </row>
-    <row r="48">
+    <row r="46" ht="14.5" customHeight="1">
+      <c r="A46" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B46" s="11" t="n"/>
+      <c r="C46" s="12" t="n"/>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="13" t="n"/>
+      <c r="F46" s="13" t="n"/>
+      <c r="G46" s="13" t="n"/>
+      <c r="H46" s="13" t="n"/>
+      <c r="I46" s="13" t="n"/>
+      <c r="J46" s="13" t="n"/>
+      <c r="K46" s="13" t="n"/>
+      <c r="L46" s="13" t="n"/>
+      <c r="M46" s="13" t="n"/>
+      <c r="N46" s="13" t="n"/>
+      <c r="O46" s="13" t="n"/>
+      <c r="P46" s="13" t="n"/>
+      <c r="Q46" s="13" t="n"/>
+      <c r="R46" s="13" t="n"/>
+      <c r="S46" s="13" t="n"/>
+      <c r="T46" s="13" t="n"/>
+      <c r="U46" s="13" t="n"/>
+      <c r="V46" s="13" t="n"/>
+      <c r="W46" s="13" t="n"/>
+      <c r="X46" s="13" t="n"/>
+      <c r="Y46" s="13" t="n"/>
+      <c r="Z46" s="13" t="n"/>
+      <c r="AA46" s="13" t="n"/>
+      <c r="AB46" s="13" t="n"/>
+      <c r="AC46" s="13" t="n"/>
+      <c r="AD46" s="13" t="n"/>
+      <c r="AE46" s="13" t="n"/>
+      <c r="AF46" s="13" t="n"/>
+      <c r="AG46" s="13" t="n"/>
+      <c r="AH46" s="13" t="n"/>
+      <c r="AI46" s="13" t="n"/>
+    </row>
+    <row r="47" ht="14.5" customHeight="1">
+      <c r="A47" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B47" s="11" t="n"/>
+      <c r="C47" s="12" t="n"/>
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="13" t="n"/>
+      <c r="F47" s="13" t="n"/>
+      <c r="G47" s="13" t="n"/>
+      <c r="H47" s="13" t="n"/>
+      <c r="I47" s="13" t="n"/>
+      <c r="J47" s="13" t="n"/>
+      <c r="K47" s="13" t="n"/>
+      <c r="L47" s="13" t="n"/>
+      <c r="M47" s="13" t="n"/>
+      <c r="N47" s="13" t="n"/>
+      <c r="O47" s="13" t="n"/>
+      <c r="P47" s="13" t="n"/>
+      <c r="Q47" s="13" t="n"/>
+      <c r="R47" s="13" t="n"/>
+      <c r="S47" s="13" t="n"/>
+      <c r="T47" s="13" t="n"/>
+      <c r="U47" s="13" t="n"/>
+      <c r="V47" s="13" t="n"/>
+      <c r="W47" s="13" t="n"/>
+      <c r="X47" s="13" t="n"/>
+      <c r="Y47" s="13" t="n"/>
+      <c r="Z47" s="13" t="n"/>
+      <c r="AA47" s="13" t="n"/>
+      <c r="AB47" s="13" t="n"/>
+      <c r="AC47" s="13" t="n"/>
+      <c r="AD47" s="13" t="n"/>
+      <c r="AE47" s="13" t="n"/>
+      <c r="AF47" s="13" t="n"/>
+      <c r="AG47" s="13" t="n"/>
+      <c r="AH47" s="13" t="n"/>
+      <c r="AI47" s="13" t="n"/>
+    </row>
+    <row r="48" ht="14.5" customHeight="1">
       <c r="A48" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B48" s="11" t="n"/>
       <c r="C48" s="12" t="n"/>
@@ -2882,9 +3123,9 @@
       <c r="AH48" s="13" t="n"/>
       <c r="AI48" s="13" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" ht="14.5" customHeight="1">
       <c r="A49" s="11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B49" s="11" t="n"/>
       <c r="C49" s="12" t="n"/>
@@ -2921,308 +3162,923 @@
       <c r="AH49" s="13" t="n"/>
       <c r="AI49" s="13" t="n"/>
     </row>
-    <row r="50">
-      <c r="A50" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="12" t="n"/>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="13" t="n"/>
-      <c r="F50" s="13" t="n"/>
-      <c r="G50" s="13" t="n"/>
-      <c r="H50" s="13" t="n"/>
-      <c r="I50" s="13" t="n"/>
-      <c r="J50" s="13" t="n"/>
-      <c r="K50" s="13" t="n"/>
-      <c r="L50" s="13" t="n"/>
-      <c r="M50" s="13" t="n"/>
-      <c r="N50" s="13" t="n"/>
-      <c r="O50" s="13" t="n"/>
-      <c r="P50" s="13" t="n"/>
-      <c r="Q50" s="13" t="n"/>
-      <c r="R50" s="13" t="n"/>
-      <c r="S50" s="13" t="n"/>
-      <c r="T50" s="13" t="n"/>
-      <c r="U50" s="13" t="n"/>
-      <c r="V50" s="13" t="n"/>
-      <c r="W50" s="13" t="n"/>
-      <c r="X50" s="13" t="n"/>
-      <c r="Y50" s="13" t="n"/>
-      <c r="Z50" s="13" t="n"/>
-      <c r="AA50" s="13" t="n"/>
-      <c r="AB50" s="13" t="n"/>
-      <c r="AC50" s="13" t="n"/>
-      <c r="AD50" s="13" t="n"/>
-      <c r="AE50" s="13" t="n"/>
-      <c r="AF50" s="13" t="n"/>
-      <c r="AG50" s="13" t="n"/>
-      <c r="AH50" s="13" t="n"/>
-      <c r="AI50" s="13" t="n"/>
-    </row>
     <row r="51">
-      <c r="A51" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="B51" s="11" t="n"/>
-      <c r="C51" s="12" t="n"/>
-      <c r="D51" s="11" t="n"/>
-      <c r="E51" s="13" t="n"/>
-      <c r="F51" s="13" t="n"/>
-      <c r="G51" s="13" t="n"/>
-      <c r="H51" s="13" t="n"/>
-      <c r="I51" s="13" t="n"/>
-      <c r="J51" s="13" t="n"/>
-      <c r="K51" s="13" t="n"/>
-      <c r="L51" s="13" t="n"/>
-      <c r="M51" s="13" t="n"/>
-      <c r="N51" s="13" t="n"/>
-      <c r="O51" s="13" t="n"/>
-      <c r="P51" s="13" t="n"/>
-      <c r="Q51" s="13" t="n"/>
-      <c r="R51" s="13" t="n"/>
-      <c r="S51" s="13" t="n"/>
-      <c r="T51" s="13" t="n"/>
-      <c r="U51" s="13" t="n"/>
-      <c r="V51" s="13" t="n"/>
-      <c r="W51" s="13" t="n"/>
-      <c r="X51" s="13" t="n"/>
-      <c r="Y51" s="13" t="n"/>
-      <c r="Z51" s="13" t="n"/>
-      <c r="AA51" s="13" t="n"/>
-      <c r="AB51" s="13" t="n"/>
-      <c r="AC51" s="13" t="n"/>
-      <c r="AD51" s="13" t="n"/>
-      <c r="AE51" s="13" t="n"/>
-      <c r="AF51" s="13" t="n"/>
-      <c r="AG51" s="13" t="n"/>
-      <c r="AH51" s="13" t="n"/>
-      <c r="AI51" s="13" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B52" s="11" t="n"/>
-      <c r="C52" s="12" t="n"/>
-      <c r="D52" s="11" t="n"/>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n"/>
-      <c r="G52" s="13" t="n"/>
-      <c r="H52" s="13" t="n"/>
-      <c r="I52" s="13" t="n"/>
-      <c r="J52" s="13" t="n"/>
-      <c r="K52" s="13" t="n"/>
-      <c r="L52" s="13" t="n"/>
-      <c r="M52" s="13" t="n"/>
-      <c r="N52" s="13" t="n"/>
-      <c r="O52" s="13" t="n"/>
-      <c r="P52" s="13" t="n"/>
-      <c r="Q52" s="13" t="n"/>
-      <c r="R52" s="13" t="n"/>
-      <c r="S52" s="13" t="n"/>
-      <c r="T52" s="13" t="n"/>
-      <c r="U52" s="13" t="n"/>
-      <c r="V52" s="13" t="n"/>
-      <c r="W52" s="13" t="n"/>
-      <c r="X52" s="13" t="n"/>
-      <c r="Y52" s="13" t="n"/>
-      <c r="Z52" s="13" t="n"/>
-      <c r="AA52" s="13" t="n"/>
-      <c r="AB52" s="13" t="n"/>
-      <c r="AC52" s="13" t="n"/>
-      <c r="AD52" s="13" t="n"/>
-      <c r="AE52" s="13" t="n"/>
-      <c r="AF52" s="13" t="n"/>
-      <c r="AG52" s="13" t="n"/>
-      <c r="AH52" s="13" t="n"/>
-      <c r="AI52" s="13" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="20" t="inlineStr">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>TOTAL DAILY
+CREWS MANPOWER</t>
+        </is>
+      </c>
+      <c r="B51" s="43" t="n"/>
+      <c r="C51" s="44" t="n"/>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>SHIFT</t>
+        </is>
+      </c>
+      <c r="E51" s="7">
+        <f>E3</f>
+        <v/>
+      </c>
+      <c r="F51" s="7">
+        <f>F3</f>
+        <v/>
+      </c>
+      <c r="G51" s="7">
+        <f>G3</f>
+        <v/>
+      </c>
+      <c r="H51" s="7">
+        <f>H3</f>
+        <v/>
+      </c>
+      <c r="I51" s="7">
+        <f>I3</f>
+        <v/>
+      </c>
+      <c r="J51" s="7">
+        <f>J3</f>
+        <v/>
+      </c>
+      <c r="K51" s="7">
+        <f>K3</f>
+        <v/>
+      </c>
+      <c r="L51" s="7">
+        <f>L3</f>
+        <v/>
+      </c>
+      <c r="M51" s="7">
+        <f>M3</f>
+        <v/>
+      </c>
+      <c r="N51" s="7">
+        <f>N3</f>
+        <v/>
+      </c>
+      <c r="O51" s="7">
+        <f>O3</f>
+        <v/>
+      </c>
+      <c r="P51" s="7">
+        <f>P3</f>
+        <v/>
+      </c>
+      <c r="Q51" s="7">
+        <f>Q3</f>
+        <v/>
+      </c>
+      <c r="R51" s="7">
+        <f>R3</f>
+        <v/>
+      </c>
+      <c r="S51" s="7">
+        <f>S3</f>
+        <v/>
+      </c>
+      <c r="T51" s="7">
+        <f>T3</f>
+        <v/>
+      </c>
+      <c r="U51" s="7">
+        <f>U3</f>
+        <v/>
+      </c>
+      <c r="V51" s="7">
+        <f>V3</f>
+        <v/>
+      </c>
+      <c r="W51" s="7">
+        <f>W3</f>
+        <v/>
+      </c>
+      <c r="X51" s="7">
+        <f>X3</f>
+        <v/>
+      </c>
+      <c r="Y51" s="7">
+        <f>Y3</f>
+        <v/>
+      </c>
+      <c r="Z51" s="7">
+        <f>Z3</f>
+        <v/>
+      </c>
+      <c r="AA51" s="7">
+        <f>AA3</f>
+        <v/>
+      </c>
+      <c r="AB51" s="7">
+        <f>AB3</f>
+        <v/>
+      </c>
+      <c r="AC51" s="7">
+        <f>AC3</f>
+        <v/>
+      </c>
+      <c r="AD51" s="7">
+        <f>AD3</f>
+        <v/>
+      </c>
+      <c r="AE51" s="7">
+        <f>AE3</f>
+        <v/>
+      </c>
+      <c r="AF51" s="7">
+        <f>AF3</f>
+        <v/>
+      </c>
+      <c r="AG51" s="7">
+        <f>AG3</f>
+        <v/>
+      </c>
+      <c r="AH51" s="7">
+        <f>AH3</f>
+        <v/>
+      </c>
+      <c r="AI51" s="7">
+        <f>AI3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="13.5" customHeight="1">
+      <c r="A52" s="45" t="n"/>
+      <c r="C52" s="46" t="n"/>
+      <c r="D52" s="22" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E52" s="11">
+        <f>IF(E$4="","",COUNTIF(E6:E49,"D"))</f>
+        <v/>
+      </c>
+      <c r="F52" s="11">
+        <f>IF(F$4="","",COUNTIF(F6:F49,"D"))</f>
+        <v/>
+      </c>
+      <c r="G52" s="11">
+        <f>IF(G$4="","",COUNTIF(G6:G49,"D"))</f>
+        <v/>
+      </c>
+      <c r="H52" s="11">
+        <f>IF(H$4="","",COUNTIF(H6:H49,"D"))</f>
+        <v/>
+      </c>
+      <c r="I52" s="11">
+        <f>IF(I$4="","",COUNTIF(I6:I49,"D"))</f>
+        <v/>
+      </c>
+      <c r="J52" s="11">
+        <f>IF(J$4="","",COUNTIF(J6:J49,"D"))</f>
+        <v/>
+      </c>
+      <c r="K52" s="11">
+        <f>IF(K$4="","",COUNTIF(K6:K49,"D"))</f>
+        <v/>
+      </c>
+      <c r="L52" s="11">
+        <f>IF(L$4="","",COUNTIF(L6:L49,"D"))</f>
+        <v/>
+      </c>
+      <c r="M52" s="11">
+        <f>IF(M$4="","",COUNTIF(M6:M49,"D"))</f>
+        <v/>
+      </c>
+      <c r="N52" s="11">
+        <f>IF(N$4="","",COUNTIF(N6:N49,"D"))</f>
+        <v/>
+      </c>
+      <c r="O52" s="11">
+        <f>IF(O$4="","",COUNTIF(O6:O49,"D"))</f>
+        <v/>
+      </c>
+      <c r="P52" s="11">
+        <f>IF(P$4="","",COUNTIF(P6:P49,"D"))</f>
+        <v/>
+      </c>
+      <c r="Q52" s="11">
+        <f>IF(Q$4="","",COUNTIF(Q6:Q49,"D"))</f>
+        <v/>
+      </c>
+      <c r="R52" s="11">
+        <f>IF(R$4="","",COUNTIF(R6:R49,"D"))</f>
+        <v/>
+      </c>
+      <c r="S52" s="11">
+        <f>IF(S$4="","",COUNTIF(S6:S49,"D"))</f>
+        <v/>
+      </c>
+      <c r="T52" s="11">
+        <f>IF(T$4="","",COUNTIF(T6:T49,"D"))</f>
+        <v/>
+      </c>
+      <c r="U52" s="11">
+        <f>IF(U$4="","",COUNTIF(U6:U49,"D"))</f>
+        <v/>
+      </c>
+      <c r="V52" s="11">
+        <f>IF(V$4="","",COUNTIF(V6:V49,"D"))</f>
+        <v/>
+      </c>
+      <c r="W52" s="11">
+        <f>IF(W$4="","",COUNTIF(W6:W49,"D"))</f>
+        <v/>
+      </c>
+      <c r="X52" s="11">
+        <f>IF(X$4="","",COUNTIF(X6:X49,"D"))</f>
+        <v/>
+      </c>
+      <c r="Y52" s="11">
+        <f>IF(Y$4="","",COUNTIF(Y6:Y49,"D"))</f>
+        <v/>
+      </c>
+      <c r="Z52" s="11">
+        <f>IF(Z$4="","",COUNTIF(Z6:Z49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AA52" s="11">
+        <f>IF(AA$4="","",COUNTIF(AA6:AA49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AB52" s="11">
+        <f>IF(AB$4="","",COUNTIF(AB6:AB49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AC52" s="11">
+        <f>IF(AC$4="","",COUNTIF(AC6:AC49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AD52" s="11">
+        <f>IF(AD$4="","",COUNTIF(AD6:AD49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AE52" s="11">
+        <f>IF(AE$4="","",COUNTIF(AE6:AE49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AF52" s="11">
+        <f>IF(AF$4="","",COUNTIF(AF6:AF49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AG52" s="11">
+        <f>IF(AG$4="","",COUNTIF(AG6:AG49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AH52" s="11">
+        <f>IF(AH$4="","",COUNTIF(AH6:AH49,"D"))</f>
+        <v/>
+      </c>
+      <c r="AI52" s="11">
+        <f>IF(AI$4="","",COUNTIF(AI6:AI49,"D"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="13.5" customHeight="1">
+      <c r="A53" s="45" t="n"/>
+      <c r="C53" s="46" t="n"/>
+      <c r="D53" s="23" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="E53" s="11">
+        <f>IF(E$4="","",COUNTIF(E6:E49,"T"))</f>
+        <v/>
+      </c>
+      <c r="F53" s="11">
+        <f>IF(F$4="","",COUNTIF(F6:F49,"T"))</f>
+        <v/>
+      </c>
+      <c r="G53" s="11">
+        <f>IF(G$4="","",COUNTIF(G6:G49,"T"))</f>
+        <v/>
+      </c>
+      <c r="H53" s="11">
+        <f>IF(H$4="","",COUNTIF(H6:H49,"T"))</f>
+        <v/>
+      </c>
+      <c r="I53" s="11">
+        <f>IF(I$4="","",COUNTIF(I6:I49,"T"))</f>
+        <v/>
+      </c>
+      <c r="J53" s="11">
+        <f>IF(J$4="","",COUNTIF(J6:J49,"T"))</f>
+        <v/>
+      </c>
+      <c r="K53" s="11">
+        <f>IF(K$4="","",COUNTIF(K6:K49,"T"))</f>
+        <v/>
+      </c>
+      <c r="L53" s="11">
+        <f>IF(L$4="","",COUNTIF(L6:L49,"T"))</f>
+        <v/>
+      </c>
+      <c r="M53" s="11">
+        <f>IF(M$4="","",COUNTIF(M6:M49,"T"))</f>
+        <v/>
+      </c>
+      <c r="N53" s="11">
+        <f>IF(N$4="","",COUNTIF(N6:N49,"T"))</f>
+        <v/>
+      </c>
+      <c r="O53" s="11">
+        <f>IF(O$4="","",COUNTIF(O6:O49,"T"))</f>
+        <v/>
+      </c>
+      <c r="P53" s="11">
+        <f>IF(P$4="","",COUNTIF(P6:P49,"T"))</f>
+        <v/>
+      </c>
+      <c r="Q53" s="11">
+        <f>IF(Q$4="","",COUNTIF(Q6:Q49,"T"))</f>
+        <v/>
+      </c>
+      <c r="R53" s="11">
+        <f>IF(R$4="","",COUNTIF(R6:R49,"T"))</f>
+        <v/>
+      </c>
+      <c r="S53" s="11">
+        <f>IF(S$4="","",COUNTIF(S6:S49,"T"))</f>
+        <v/>
+      </c>
+      <c r="T53" s="11">
+        <f>IF(T$4="","",COUNTIF(T6:T49,"T"))</f>
+        <v/>
+      </c>
+      <c r="U53" s="11">
+        <f>IF(U$4="","",COUNTIF(U6:U49,"T"))</f>
+        <v/>
+      </c>
+      <c r="V53" s="11">
+        <f>IF(V$4="","",COUNTIF(V6:V49,"T"))</f>
+        <v/>
+      </c>
+      <c r="W53" s="11">
+        <f>IF(W$4="","",COUNTIF(W6:W49,"T"))</f>
+        <v/>
+      </c>
+      <c r="X53" s="11">
+        <f>IF(X$4="","",COUNTIF(X6:X49,"T"))</f>
+        <v/>
+      </c>
+      <c r="Y53" s="11">
+        <f>IF(Y$4="","",COUNTIF(Y6:Y49,"T"))</f>
+        <v/>
+      </c>
+      <c r="Z53" s="11">
+        <f>IF(Z$4="","",COUNTIF(Z6:Z49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AA53" s="11">
+        <f>IF(AA$4="","",COUNTIF(AA6:AA49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AB53" s="11">
+        <f>IF(AB$4="","",COUNTIF(AB6:AB49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AC53" s="11">
+        <f>IF(AC$4="","",COUNTIF(AC6:AC49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AD53" s="11">
+        <f>IF(AD$4="","",COUNTIF(AD6:AD49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AE53" s="11">
+        <f>IF(AE$4="","",COUNTIF(AE6:AE49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AF53" s="11">
+        <f>IF(AF$4="","",COUNTIF(AF6:AF49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AG53" s="11">
+        <f>IF(AG$4="","",COUNTIF(AG6:AG49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AH53" s="11">
+        <f>IF(AH$4="","",COUNTIF(AH6:AH49,"T"))</f>
+        <v/>
+      </c>
+      <c r="AI53" s="11">
+        <f>IF(AI$4="","",COUNTIF(AI6:AI49,"T"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="13.5" customHeight="1">
+      <c r="A54" s="47" t="n"/>
+      <c r="B54" s="48" t="n"/>
+      <c r="C54" s="49" t="n"/>
+      <c r="D54" s="24" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E54" s="11">
+        <f>IF(E$4="","",COUNTIF(E6:E49,"G"))</f>
+        <v/>
+      </c>
+      <c r="F54" s="11">
+        <f>IF(F$4="","",COUNTIF(F6:F49,"G"))</f>
+        <v/>
+      </c>
+      <c r="G54" s="11">
+        <f>IF(G$4="","",COUNTIF(G6:G49,"G"))</f>
+        <v/>
+      </c>
+      <c r="H54" s="11">
+        <f>IF(H$4="","",COUNTIF(H6:H49,"G"))</f>
+        <v/>
+      </c>
+      <c r="I54" s="11">
+        <f>IF(I$4="","",COUNTIF(I6:I49,"G"))</f>
+        <v/>
+      </c>
+      <c r="J54" s="11">
+        <f>IF(J$4="","",COUNTIF(J6:J49,"G"))</f>
+        <v/>
+      </c>
+      <c r="K54" s="11">
+        <f>IF(K$4="","",COUNTIF(K6:K49,"G"))</f>
+        <v/>
+      </c>
+      <c r="L54" s="11">
+        <f>IF(L$4="","",COUNTIF(L6:L49,"G"))</f>
+        <v/>
+      </c>
+      <c r="M54" s="11">
+        <f>IF(M$4="","",COUNTIF(M6:M49,"G"))</f>
+        <v/>
+      </c>
+      <c r="N54" s="11">
+        <f>IF(N$4="","",COUNTIF(N6:N49,"G"))</f>
+        <v/>
+      </c>
+      <c r="O54" s="11">
+        <f>IF(O$4="","",COUNTIF(O6:O49,"G"))</f>
+        <v/>
+      </c>
+      <c r="P54" s="11">
+        <f>IF(P$4="","",COUNTIF(P6:P49,"G"))</f>
+        <v/>
+      </c>
+      <c r="Q54" s="11">
+        <f>IF(Q$4="","",COUNTIF(Q6:Q49,"G"))</f>
+        <v/>
+      </c>
+      <c r="R54" s="11">
+        <f>IF(R$4="","",COUNTIF(R6:R49,"G"))</f>
+        <v/>
+      </c>
+      <c r="S54" s="11">
+        <f>IF(S$4="","",COUNTIF(S6:S49,"G"))</f>
+        <v/>
+      </c>
+      <c r="T54" s="11">
+        <f>IF(T$4="","",COUNTIF(T6:T49,"G"))</f>
+        <v/>
+      </c>
+      <c r="U54" s="11">
+        <f>IF(U$4="","",COUNTIF(U6:U49,"G"))</f>
+        <v/>
+      </c>
+      <c r="V54" s="11">
+        <f>IF(V$4="","",COUNTIF(V6:V49,"G"))</f>
+        <v/>
+      </c>
+      <c r="W54" s="11">
+        <f>IF(W$4="","",COUNTIF(W6:W49,"G"))</f>
+        <v/>
+      </c>
+      <c r="X54" s="11">
+        <f>IF(X$4="","",COUNTIF(X6:X49,"G"))</f>
+        <v/>
+      </c>
+      <c r="Y54" s="11">
+        <f>IF(Y$4="","",COUNTIF(Y6:Y49,"G"))</f>
+        <v/>
+      </c>
+      <c r="Z54" s="11">
+        <f>IF(Z$4="","",COUNTIF(Z6:Z49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AA54" s="11">
+        <f>IF(AA$4="","",COUNTIF(AA6:AA49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AB54" s="11">
+        <f>IF(AB$4="","",COUNTIF(AB6:AB49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AC54" s="11">
+        <f>IF(AC$4="","",COUNTIF(AC6:AC49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AD54" s="11">
+        <f>IF(AD$4="","",COUNTIF(AD6:AD49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AE54" s="11">
+        <f>IF(AE$4="","",COUNTIF(AE6:AE49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AF54" s="11">
+        <f>IF(AF$4="","",COUNTIF(AF6:AF49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AG54" s="11">
+        <f>IF(AG$4="","",COUNTIF(AG6:AG49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AH54" s="11">
+        <f>IF(AH$4="","",COUNTIF(AH6:AH49,"G"))</f>
+        <v/>
+      </c>
+      <c r="AI54" s="11">
+        <f>IF(AI$4="","",COUNTIF(AI6:AI49,"G"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="13.5" customHeight="1">
+      <c r="A55" s="21" t="n"/>
+      <c r="B55" s="21" t="n"/>
+      <c r="C55" s="21" t="n"/>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>TOT</t>
+        </is>
+      </c>
+      <c r="E55" s="13">
+        <f>IF(E$4="","",SUM(E52:E54))</f>
+        <v/>
+      </c>
+      <c r="F55" s="13">
+        <f>IF(F$4="","",SUM(F52:F54))</f>
+        <v/>
+      </c>
+      <c r="G55" s="13">
+        <f>IF(G$4="","",SUM(G52:G54))</f>
+        <v/>
+      </c>
+      <c r="H55" s="13">
+        <f>IF(H$4="","",SUM(H52:H54))</f>
+        <v/>
+      </c>
+      <c r="I55" s="13">
+        <f>IF(I$4="","",SUM(I52:I54))</f>
+        <v/>
+      </c>
+      <c r="J55" s="13">
+        <f>IF(J$4="","",SUM(J52:J54))</f>
+        <v/>
+      </c>
+      <c r="K55" s="13">
+        <f>IF(K$4="","",SUM(K52:K54))</f>
+        <v/>
+      </c>
+      <c r="L55" s="13">
+        <f>IF(L$4="","",SUM(L52:L54))</f>
+        <v/>
+      </c>
+      <c r="M55" s="13">
+        <f>IF(M$4="","",SUM(M52:M54))</f>
+        <v/>
+      </c>
+      <c r="N55" s="13">
+        <f>IF(N$4="","",SUM(N52:N54))</f>
+        <v/>
+      </c>
+      <c r="O55" s="13">
+        <f>IF(O$4="","",SUM(O52:O54))</f>
+        <v/>
+      </c>
+      <c r="P55" s="13">
+        <f>IF(P$4="","",SUM(P52:P54))</f>
+        <v/>
+      </c>
+      <c r="Q55" s="13">
+        <f>IF(Q$4="","",SUM(Q52:Q54))</f>
+        <v/>
+      </c>
+      <c r="R55" s="13">
+        <f>IF(R$4="","",SUM(R52:R54))</f>
+        <v/>
+      </c>
+      <c r="S55" s="13">
+        <f>IF(S$4="","",SUM(S52:S54))</f>
+        <v/>
+      </c>
+      <c r="T55" s="13">
+        <f>IF(T$4="","",SUM(T52:T54))</f>
+        <v/>
+      </c>
+      <c r="U55" s="13">
+        <f>IF(U$4="","",SUM(U52:U54))</f>
+        <v/>
+      </c>
+      <c r="V55" s="13">
+        <f>IF(V$4="","",SUM(V52:V54))</f>
+        <v/>
+      </c>
+      <c r="W55" s="13">
+        <f>IF(W$4="","",SUM(W52:W54))</f>
+        <v/>
+      </c>
+      <c r="X55" s="13">
+        <f>IF(X$4="","",SUM(X52:X54))</f>
+        <v/>
+      </c>
+      <c r="Y55" s="13">
+        <f>IF(Y$4="","",SUM(Y52:Y54))</f>
+        <v/>
+      </c>
+      <c r="Z55" s="13">
+        <f>IF(Z$4="","",SUM(Z52:Z54))</f>
+        <v/>
+      </c>
+      <c r="AA55" s="13">
+        <f>IF(AA$4="","",SUM(AA52:AA54))</f>
+        <v/>
+      </c>
+      <c r="AB55" s="13">
+        <f>IF(AB$4="","",SUM(AB52:AB54))</f>
+        <v/>
+      </c>
+      <c r="AC55" s="13">
+        <f>IF(AC$4="","",SUM(AC52:AC54))</f>
+        <v/>
+      </c>
+      <c r="AD55" s="13">
+        <f>IF(AD$4="","",SUM(AD52:AD54))</f>
+        <v/>
+      </c>
+      <c r="AE55" s="13">
+        <f>IF(AE$4="","",SUM(AE52:AE54))</f>
+        <v/>
+      </c>
+      <c r="AF55" s="13">
+        <f>IF(AF$4="","",SUM(AF52:AF54))</f>
+        <v/>
+      </c>
+      <c r="AG55" s="13">
+        <f>IF(AG$4="","",SUM(AG52:AG54))</f>
+        <v/>
+      </c>
+      <c r="AH55" s="13">
+        <f>IF(AH$4="","",SUM(AH52:AH54))</f>
+        <v/>
+      </c>
+      <c r="AI55" s="13">
+        <f>IF(AI$4="","",SUM(AI52:AI54))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>SHIFT TIMES</t>
+        </is>
+      </c>
+      <c r="F57" s="25" t="inlineStr">
         <is>
           <t>CODE LEGEND</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="21" t="inlineStr">
+    <row r="58" ht="14" customHeight="1">
+      <c r="B58" s="26" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B56" s="22" t="inlineStr">
+      <c r="C58" s="27" t="inlineStr">
+        <is>
+          <t>DAY (07:00 - 15:00)</t>
+        </is>
+      </c>
+      <c r="F58" s="22" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G58" s="50" t="n"/>
+      <c r="H58" s="28" t="inlineStr">
         <is>
           <t>DAY</t>
         </is>
       </c>
-      <c r="C56" s="23" t="inlineStr">
+      <c r="J58" s="23" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="D56" s="22" t="inlineStr">
+      <c r="K58" s="50" t="n"/>
+      <c r="L58" s="28" t="inlineStr">
         <is>
           <t>TWILIGHT</t>
         </is>
       </c>
-      <c r="E56" s="24" t="inlineStr">
+      <c r="N58" s="24" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="F56" s="22" t="inlineStr">
+      <c r="O58" s="50" t="n"/>
+      <c r="P58" s="28" t="inlineStr">
         <is>
           <t>GRAVEYARD</t>
         </is>
       </c>
-      <c r="G56" s="25" t="inlineStr">
+      <c r="R58" s="29" t="inlineStr">
         <is>
           <t>TR</t>
         </is>
       </c>
-      <c r="H56" s="22" t="inlineStr">
+      <c r="S58" s="50" t="n"/>
+      <c r="T58" s="28" t="inlineStr">
         <is>
           <t>TRAINING</t>
         </is>
       </c>
-      <c r="I56" s="26" t="inlineStr">
+      <c r="V58" s="30" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="J56" s="22" t="inlineStr">
+      <c r="W58" s="50" t="n"/>
+      <c r="X58" s="28" t="inlineStr">
         <is>
           <t>VACATION</t>
         </is>
       </c>
-      <c r="K56" s="27" t="inlineStr">
+      <c r="Z58" s="31" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="L56" s="22" t="inlineStr">
+      <c r="AA58" s="50" t="n"/>
+      <c r="AB58" s="28" t="inlineStr">
         <is>
           <t>REST/RDO</t>
         </is>
       </c>
-      <c r="M56" s="28" t="inlineStr">
+      <c r="AD58" s="32" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="N56" s="22" t="inlineStr">
+      <c r="AE58" s="50" t="n"/>
+      <c r="AF58" s="28" t="inlineStr">
         <is>
           <t>ABSENT</t>
         </is>
       </c>
-      <c r="O56" s="29" t="inlineStr">
+    </row>
+    <row r="59" ht="14" customHeight="1">
+      <c r="B59" s="33" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C59" s="27" t="inlineStr">
+        <is>
+          <t>TWI (15:00 - 23:00)</t>
+        </is>
+      </c>
+      <c r="F59" s="34" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="P56" s="22" t="inlineStr">
+      <c r="G59" s="50" t="n"/>
+      <c r="H59" s="28" t="inlineStr">
         <is>
           <t>HOLIDAY</t>
         </is>
       </c>
-      <c r="Q56" s="30" t="inlineStr">
+      <c r="J59" s="35" t="inlineStr">
         <is>
           <t>OT</t>
         </is>
       </c>
-      <c r="R56" s="22" t="inlineStr">
+      <c r="K59" s="50" t="n"/>
+      <c r="L59" s="28" t="inlineStr">
         <is>
           <t>OVERTIME</t>
         </is>
       </c>
-      <c r="S56" s="31" t="inlineStr">
+      <c r="N59" s="36" t="inlineStr">
         <is>
           <t>OS</t>
         </is>
       </c>
-      <c r="T56" s="22" t="inlineStr">
+      <c r="O59" s="50" t="n"/>
+      <c r="P59" s="28" t="inlineStr">
         <is>
           <t>OUTSTATION</t>
         </is>
       </c>
-      <c r="U56" s="32" t="inlineStr">
+      <c r="R59" s="37" t="inlineStr">
         <is>
           <t>S/L</t>
         </is>
       </c>
-      <c r="V56" s="22" t="inlineStr">
+      <c r="S59" s="50" t="n"/>
+      <c r="T59" s="28" t="inlineStr">
         <is>
           <t>SICK LEAVE</t>
         </is>
       </c>
-      <c r="W56" s="33" t="inlineStr">
+      <c r="V59" s="38" t="inlineStr">
         <is>
           <t>C/T</t>
         </is>
       </c>
-      <c r="X56" s="22" t="inlineStr">
+      <c r="W59" s="50" t="n"/>
+      <c r="X59" s="28" t="inlineStr">
         <is>
           <t>COMP TIME</t>
         </is>
       </c>
-      <c r="Y56" s="34" t="inlineStr">
+      <c r="Z59" s="39" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="Z56" s="22" t="inlineStr">
+      <c r="AA59" s="50" t="n"/>
+      <c r="AB59" s="28" t="inlineStr">
         <is>
           <t>LATE/LEAVE</t>
         </is>
       </c>
-      <c r="AA56" s="35" t="inlineStr">
+      <c r="AD59" s="40" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="AB56" s="22" t="inlineStr">
+      <c r="AE59" s="50" t="n"/>
+      <c r="AF59" s="28" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>PREPARED BY:</t>
-        </is>
-      </c>
-      <c r="C59" s="36" t="n"/>
-      <c r="D59" s="37" t="n"/>
-      <c r="E59" s="37" t="n"/>
-      <c r="F59" s="37" t="n"/>
-      <c r="G59" s="37" t="n"/>
-      <c r="H59" s="37" t="n"/>
-      <c r="T59" s="4" t="inlineStr">
-        <is>
-          <t>APPROVED BY:</t>
-        </is>
-      </c>
-      <c r="V59" s="36" t="n"/>
-      <c r="W59" s="37" t="n"/>
-      <c r="X59" s="37" t="n"/>
-      <c r="Y59" s="37" t="n"/>
-      <c r="Z59" s="37" t="n"/>
-      <c r="AA59" s="37" t="n"/>
+    <row r="60" ht="14" customHeight="1">
+      <c r="B60" s="41" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C60" s="27" t="inlineStr">
+        <is>
+          <t>GRV (23:00 - 07:00)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="40">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E2:AI2"/>
+    <mergeCell ref="AB58:AC58"/>
+    <mergeCell ref="C58:D58"/>
+    <mergeCell ref="E1:AE1"/>
+    <mergeCell ref="V58:W58"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="R59:S59"/>
+    <mergeCell ref="AF1:AI1"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="T58:U58"/>
+    <mergeCell ref="AD59:AE59"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A51:C54"/>
+    <mergeCell ref="P59:Q59"/>
+    <mergeCell ref="T59:U59"/>
+    <mergeCell ref="V59:W59"/>
+    <mergeCell ref="AB59:AC59"/>
+    <mergeCell ref="N58:O58"/>
+    <mergeCell ref="Z58:AA58"/>
+    <mergeCell ref="C59:D59"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="V59:AA59"/>
-    <mergeCell ref="E2:AC2"/>
-    <mergeCell ref="E1:Y1"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="Z1:AC1"/>
-    <mergeCell ref="C59:H59"/>
-    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="L58:M58"/>
+    <mergeCell ref="X58:Y58"/>
+    <mergeCell ref="AF59:AG59"/>
+    <mergeCell ref="AF58:AG58"/>
+    <mergeCell ref="N59:O59"/>
+    <mergeCell ref="F58:G58"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="L59:M59"/>
+    <mergeCell ref="X59:Y59"/>
+    <mergeCell ref="P58:Q58"/>
+    <mergeCell ref="Z59:AA59"/>
+    <mergeCell ref="R58:S58"/>
+    <mergeCell ref="J58:K58"/>
+    <mergeCell ref="AD58:AE58"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:AI17">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -3271,7 +4127,7 @@
       <formula>AND(E$4&lt;&gt;"",OR(E$3="Fri",E$3="Sat"))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E20:AI31">
+  <conditionalFormatting sqref="E19:AI30">
     <cfRule type="cellIs" priority="16" operator="equal" dxfId="0">
       <formula>"D"</formula>
     </cfRule>
@@ -3318,7 +4174,7 @@
       <formula>AND(E$4&lt;&gt;"",OR(E$3="Fri",E$3="Sat"))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E34:AI45">
+  <conditionalFormatting sqref="E32:AI43">
     <cfRule type="cellIs" priority="31" operator="equal" dxfId="0">
       <formula>"D"</formula>
     </cfRule>
@@ -3365,7 +4221,7 @@
       <formula>AND(E$4&lt;&gt;"",OR(E$3="Fri",E$3="Sat"))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E48:AI52">
+  <conditionalFormatting sqref="E45:AI49">
     <cfRule type="cellIs" priority="46" operator="equal" dxfId="0">
       <formula>"D"</formula>
     </cfRule>
@@ -3412,7 +4268,8 @@
       <formula>AND(E$4&lt;&gt;"",OR(E$3="Fri",E$3="Sat"))</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>